<commit_message>
manual and docs changes
</commit_message>
<xml_diff>
--- a/packages/core/src/state-testing-and-appendices/SanityCheck_DoLLMsUnderstandRepresentationOfOurDiagrams.xlsx
+++ b/packages/core/src/state-testing-and-appendices/SanityCheck_DoLLMsUnderstandRepresentationOfOurDiagrams.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PETO\Desktop\Workspaces\Markup and docs\State-Diagrams-Bc-Thesis\content\appendices\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PETO\Desktop\Workspaces\HTML\VsCodeIDEs\react-diagrams-vscode\packages\core\src\state-testing-and-appendices\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C3E117-5CFD-4C04-8308-CAEF9EDF3A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -412,6 +412,9 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -424,16 +427,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1943,7 +1943,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="20" t="s">
         <v>28</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1988,10 +1988,10 @@
         <f>(LEFT(B3,FIND("/",B3)-1)/MID(B3,FIND("/",B3)+1,LEN(B3)))*0.1+(LEFT(C3,FIND("/",C3)-1)/MID(C3,FIND("/",C3)+1,LEN(C3)))*0.1+(LEFT(D3,FIND("/",D3)-1)/MID(D3,FIND("/",D3)+1,LEN(D3)))*0.25+(LEFT(E3,FIND("/",E3)-1)/MID(E3,FIND("/",E3)+1,LEN(E3)))*0.55</f>
         <v>1</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="25">
         <f>AVERAGE(F3,F4,F5,F6)</f>
         <v>0.97937500000000011</v>
       </c>
@@ -2016,8 +2016,8 @@
         <f t="shared" ref="F4:F16" si="0">(LEFT(B4,FIND("/",B4)-1)/MID(B4,FIND("/",B4)+1,LEN(B4)))*0.1+(LEFT(C4,FIND("/",C4)-1)/MID(C4,FIND("/",C4)+1,LEN(C4)))*0.1+(LEFT(D4,FIND("/",D4)-1)/MID(D4,FIND("/",D4)+1,LEN(D4)))*0.25+(LEFT(E4,FIND("/",E4)-1)/MID(E4,FIND("/",E4)+1,LEN(E4)))*0.55</f>
         <v>1</v>
       </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="25"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
@@ -2039,8 +2039,8 @@
         <f t="shared" si="0"/>
         <v>0.94500000000000006</v>
       </c>
-      <c r="G5" s="21"/>
-      <c r="H5" s="25"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
@@ -2062,8 +2062,8 @@
         <f t="shared" si="0"/>
         <v>0.97249999999999992</v>
       </c>
-      <c r="G6" s="22"/>
-      <c r="H6" s="25"/>
+      <c r="G6" s="23"/>
+      <c r="H6" s="26"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
@@ -2085,10 +2085,10 @@
         <f t="shared" si="0"/>
         <v>0.79361111111111116</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="27">
         <f>AVERAGE(F7,F8,F9,F10,F11,F12)</f>
         <v>0.75356481481481496</v>
       </c>
@@ -2113,8 +2113,8 @@
         <f t="shared" si="0"/>
         <v>0.64250000000000007</v>
       </c>
-      <c r="G8" s="21"/>
-      <c r="H8" s="25"/>
+      <c r="G8" s="22"/>
+      <c r="H8" s="26"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -2136,8 +2136,8 @@
         <f t="shared" si="0"/>
         <v>0.75250000000000006</v>
       </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="25"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
@@ -2159,8 +2159,8 @@
         <f t="shared" si="0"/>
         <v>0.8486111111111112</v>
       </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="25"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="26"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
@@ -2182,8 +2182,8 @@
         <f t="shared" si="0"/>
         <v>0.73166666666666669</v>
       </c>
-      <c r="G11" s="21"/>
-      <c r="H11" s="25"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="26"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
@@ -2205,8 +2205,8 @@
         <f t="shared" si="0"/>
         <v>0.75250000000000006</v>
       </c>
-      <c r="G12" s="22"/>
-      <c r="H12" s="25"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="26"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
@@ -2228,10 +2228,10 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G13" s="23" t="s">
+      <c r="G13" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="27">
         <f>AVERAGE(F13,F14,F15,F16)</f>
         <v>1</v>
       </c>
@@ -2256,8 +2256,8 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G14" s="21"/>
-      <c r="H14" s="25"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
@@ -2279,8 +2279,8 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G15" s="21"/>
-      <c r="H15" s="25"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
@@ -2302,8 +2302,8 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G16" s="22"/>
-      <c r="H16" s="25"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="18" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E18" s="18" t="s">

</xml_diff>